<commit_message>
Modified posted, updated and reviewed  dates tests
</commit_message>
<xml_diff>
--- a/test-data/dates-data.xlsx
+++ b/test-data/dates-data.xlsx
@@ -8,17 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A0D6390-A6C2-0948-84DC-9E2FAAF688D4}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2336627C-7E37-5C4A-B32C-CF99B8132AE2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4800" yWindow="460" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
+    <workbookView xWindow="4760" yWindow="3240" windowWidth="30280" windowHeight="15240" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_updated_date" sheetId="5" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="6" r:id="rId2"/>
-    <sheet name="pages_without_updated_date" sheetId="2" r:id="rId3"/>
+    <sheet name="pages_with_reviewed_date" sheetId="10" r:id="rId2"/>
+    <sheet name="pages_with_posted_date" sheetId="7" r:id="rId3"/>
+    <sheet name="pages_without_dates" sheetId="2" r:id="rId4"/>
   </sheets>
   <calcPr calcId="181029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="59">
   <si>
     <t>path</t>
   </si>
@@ -93,21 +93,6 @@
     <t>13 de julio de 2018</t>
   </si>
   <si>
-    <t>Updated:</t>
-  </si>
-  <si>
-    <t>Actualización:</t>
-  </si>
-  <si>
-    <t>news-events/cancer-currents-blog/2019/cancer-risk-total-diet</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Blog </t>
-  </si>
-  <si>
-    <t>January 1, 2019</t>
-  </si>
-  <si>
     <t>types/retinoblastoma/patient/retinoblastoma-treatment-pdq</t>
   </si>
   <si>
@@ -123,9 +108,6 @@
     <t>espanol/tipos/retinoblastoma/paciente/tratamiento-retinoblastoma-pdq</t>
   </si>
   <si>
-    <t>dateLabel</t>
-  </si>
-  <si>
     <t>about-cancer/coping/article-no-date</t>
   </si>
   <si>
@@ -151,6 +133,78 @@
   </si>
   <si>
     <t>espanol/cancer/sobrellevar/esparticle-no-date</t>
+  </si>
+  <si>
+    <t>postedDate</t>
+  </si>
+  <si>
+    <t>news-events/cancer-currents-blog/2019/expanding-clinical-trial-eligibility-criteria</t>
+  </si>
+  <si>
+    <t>Blog Post</t>
+  </si>
+  <si>
+    <t>March 7, 2019</t>
+  </si>
+  <si>
+    <t>reviewedDate</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation</t>
+  </si>
+  <si>
+    <t>February 29, 2016</t>
+  </si>
+  <si>
+    <t>24 de agosto de 2018</t>
+  </si>
+  <si>
+    <t>espanol/tipos/seno/pro/prevencion-seno-pdq</t>
+  </si>
+  <si>
+    <t>espanol/cancer/sobrellevar/sentimientos/relajarse</t>
+  </si>
+  <si>
+    <t>29 de febrero de 2016</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/chanock-stephen</t>
+  </si>
+  <si>
+    <t>espanol/node/30/2019/vitamina-d-complemento-cancer-prevencion</t>
+  </si>
+  <si>
+    <t>9 de enero de 2019</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/duke-university</t>
+  </si>
+  <si>
+    <t>July 26, 2012</t>
+  </si>
+  <si>
+    <t>news-events/press-releases/2019/deep-learning-cervical-cancer-screening</t>
+  </si>
+  <si>
+    <t>January 10, 2019</t>
+  </si>
+  <si>
+    <t>espanol/noticias/comunicados-de-prensa/2019/aprendizaje-profundo-cancer-cuello-uterino-examenes-de</t>
+  </si>
+  <si>
+    <t>10 de enero de 2019</t>
+  </si>
+  <si>
+    <t>April 16, 2019</t>
+  </si>
+  <si>
+    <t>espanol/node/87</t>
+  </si>
+  <si>
+    <t>13 de diciembre de 2018</t>
+  </si>
+  <si>
+    <t>research/key-initiatives/ras/ras-central/discussion-forum</t>
   </si>
 </sst>
 </file>
@@ -507,17 +561,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61587B9F-5CDD-9140-AFE3-DF7999F08D55}">
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="90.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.1640625" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -528,13 +581,10 @@
         <v>4</v>
       </c>
       <c r="D1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -544,31 +594,25 @@
       <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>8</v>
       </c>
@@ -578,98 +622,83 @@
       <c r="C4" t="s">
         <v>5</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>21</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B5" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>26</v>
-      </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
         <v>5</v>
       </c>
-      <c r="D6" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D6" s="3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
+        <v>19</v>
+      </c>
+      <c r="B7" t="s">
         <v>23</v>
       </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
       <c r="C7" t="s">
-        <v>5</v>
-      </c>
-      <c r="E7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" t="s">
-        <v>18</v>
-      </c>
       <c r="B8" t="s">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
         <v>17</v>
       </c>
-      <c r="D8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E8" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="D8" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>28</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
-      </c>
-      <c r="D9" t="s">
-        <v>22</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
         <v>3</v>
@@ -677,45 +706,253 @@
       <c r="C10" t="s">
         <v>17</v>
       </c>
-      <c r="D10" t="s">
-        <v>22</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+      <c r="D10" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B11" t="s">
-        <v>28</v>
-      </c>
-      <c r="C11" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>29</v>
-      </c>
     </row>
   </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D10">
+    <sortCondition ref="B1"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4A0C097F-378B-0A4A-A088-173D7C4DAF88}">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A3FA8860-EA83-E849-ADF5-B5E0EA4AD9CC}">
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="70" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D9">
+    <sortCondition ref="B1"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7C04997D-A86B-9A4F-846B-360EEAD9270F}">
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="70" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C4" t="s">
+        <v>5</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" t="s">
+        <v>37</v>
+      </c>
+      <c r="C5" t="s">
+        <v>5</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>51</v>
+      </c>
+      <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>5</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>54</v>
+      </c>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:D9">
+    <sortCondition ref="B1"/>
+  </sortState>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC26DAC-9091-7441-904D-1932A7FF4396}">
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -737,7 +974,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -748,7 +985,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
         <v>3</v>
@@ -759,7 +996,7 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="B4" t="s">
         <v>6</v>
@@ -770,7 +1007,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -781,7 +1018,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -792,7 +1029,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B7" t="s">
         <v>3</v>

</xml_diff>

<commit_message>
refactored Simple dates tests in separate methods
</commit_message>
<xml_diff>
--- a/test-data/dates-data.xlsx
+++ b/test-data/dates-data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10414"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5B9E962-137C-9846-B40E-13F20BB7421A}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0949F852-CB7D-A448-8709-81072D8A2B41}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="38400" windowHeight="21140" activeTab="1" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_simple_dates" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
   <si>
     <t>path</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Cancer Center</t>
   </si>
   <si>
-    <t>about-cancer/coping/feelings/relaxation/dfharvard</t>
-  </si>
-  <si>
     <t>about-cancer/coping/feelings/relaxation/loukissas-jen-biography</t>
   </si>
   <si>
@@ -106,30 +103,12 @@
     <t>about-cancer/coping/feelings/relaxation/duke-university</t>
   </si>
   <si>
-    <t>July 26, 2012</t>
-  </si>
-  <si>
     <t>April 16, 2019</t>
   </si>
   <si>
-    <t>espanol/node/87</t>
-  </si>
-  <si>
-    <t>13 de diciembre de 2018</t>
-  </si>
-  <si>
     <t>research/key-initiatives/ras/ras-central/discussion-forum</t>
   </si>
   <si>
-    <t>dateStamp</t>
-  </si>
-  <si>
-    <t>dateText</t>
-  </si>
-  <si>
-    <t>dateLabel</t>
-  </si>
-  <si>
     <t>Updated:</t>
   </si>
   <si>
@@ -145,21 +124,9 @@
     <t>Posted:</t>
   </si>
   <si>
-    <t>2012-07-26T12:00:00Z</t>
-  </si>
-  <si>
-    <t>pediatric-match-infographic</t>
-  </si>
-  <si>
     <t>Infographic</t>
   </si>
   <si>
-    <t>July 24, 2017</t>
-  </si>
-  <si>
-    <t>2017-07-24T12:00:00Z</t>
-  </si>
-  <si>
     <t>2016-02-29T12:00:00Z</t>
   </si>
   <si>
@@ -175,12 +142,6 @@
     <t>2019-04-16T12:00:00Z</t>
   </si>
   <si>
-    <t>2018-12-13T12:00:00Z</t>
-  </si>
-  <si>
-    <t>about-cancer/coping/feelings/relaxation/dukeci</t>
-  </si>
-  <si>
     <t>2015-01-09T12:00:00Z</t>
   </si>
   <si>
@@ -200,6 +161,33 @@
   </si>
   <si>
     <t>Video</t>
+  </si>
+  <si>
+    <t>expectedText</t>
+  </si>
+  <si>
+    <t>expectedStamp</t>
+  </si>
+  <si>
+    <t>expectedLabel</t>
+  </si>
+  <si>
+    <t>espanol/cancer/sobrellevar/sentimientos/hoja-informativa-estres</t>
+  </si>
+  <si>
+    <t>10 de diciembre de 2012</t>
+  </si>
+  <si>
+    <t>2012-12-10T12:00:00Z</t>
+  </si>
+  <si>
+    <t>about-nci/organization/screen-to-save-infographicv</t>
+  </si>
+  <si>
+    <t>February 27, 2017</t>
+  </si>
+  <si>
+    <t>2017-02-27T12:00:00Z</t>
   </si>
 </sst>
 </file>
@@ -552,7 +540,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61587B9F-5CDD-9140-AFE3-DF7999F08D55}">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="55.6640625" bestFit="1" customWidth="1"/>
@@ -573,18 +561,18 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>33</v>
+        <v>47</v>
       </c>
       <c r="E1" t="s">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="F1" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -593,38 +581,38 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="E2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>36</v>
+        <v>29</v>
       </c>
       <c r="E3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -633,38 +621,38 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="E5" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -673,98 +661,98 @@
         <v>4</v>
       </c>
       <c r="D6" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E6" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E7" t="s">
-        <v>29</v>
+        <v>49</v>
       </c>
       <c r="F7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>6</v>
+      </c>
+      <c r="B8" t="s">
         <v>7</v>
       </c>
-      <c r="B8" t="s">
-        <v>8</v>
-      </c>
       <c r="C8" t="s">
         <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C10" t="s">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="E10" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
@@ -773,77 +761,37 @@
         <v>4</v>
       </c>
       <c r="D11" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F11" t="s">
         <v>38</v>
-      </c>
-      <c r="E11" t="s">
-        <v>26</v>
-      </c>
-      <c r="F11" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="F12" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
-        <v>6</v>
-      </c>
-      <c r="B13" t="s">
-        <v>5</v>
-      </c>
-      <c r="C13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D13" t="s">
-        <v>47</v>
-      </c>
-      <c r="E13" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" t="s">
-        <v>4</v>
-      </c>
-      <c r="D14" t="s">
-        <v>38</v>
-      </c>
-      <c r="E14" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" t="s">
-        <v>43</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F14">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F12">
     <sortCondition ref="B1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -872,7 +820,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -883,7 +831,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -894,10 +842,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -905,21 +853,21 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>54</v>
+        <v>41</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -927,10 +875,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
@@ -938,10 +886,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>57</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
         <v>4</v>

</xml_diff>

<commit_message>
Fixed Data for No dates display
</commit_message>
<xml_diff>
--- a/test-data/dates-data.xlsx
+++ b/test-data/dates-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0949F852-CB7D-A448-8709-81072D8A2B41}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6FAC28-9732-F34C-B77F-F9EB14F6658D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19140" activeTab="1" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_simple_dates" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
   <si>
     <t>path</t>
   </si>
@@ -103,12 +103,6 @@
     <t>about-cancer/coping/feelings/relaxation/duke-university</t>
   </si>
   <si>
-    <t>April 16, 2019</t>
-  </si>
-  <si>
-    <t>research/key-initiatives/ras/ras-central/discussion-forum</t>
-  </si>
-  <si>
     <t>Updated:</t>
   </si>
   <si>
@@ -139,27 +133,12 @@
     <t>Reviewed:</t>
   </si>
   <si>
-    <t>2019-04-16T12:00:00Z</t>
-  </si>
-  <si>
     <t>2015-01-09T12:00:00Z</t>
   </si>
   <si>
     <t>about-cancer/coping/feelings/relaxation/loukissas-jennifer</t>
   </si>
   <si>
-    <t>file-url-sample</t>
-  </si>
-  <si>
-    <t>File</t>
-  </si>
-  <si>
-    <t>nci-at-a-glance</t>
-  </si>
-  <si>
-    <t>gutcheck-intro-video</t>
-  </si>
-  <si>
     <t>Video</t>
   </si>
   <si>
@@ -181,23 +160,50 @@
     <t>2012-12-10T12:00:00Z</t>
   </si>
   <si>
-    <t>about-nci/organization/screen-to-save-infographicv</t>
-  </si>
-  <si>
-    <t>February 27, 2017</t>
-  </si>
-  <si>
-    <t>2017-02-27T12:00:00Z</t>
+    <t>espanol/investigacion/es-hedge-maze</t>
+  </si>
+  <si>
+    <t>about-cancer/coping/feelings/relaxation/hedge-maze</t>
+  </si>
+  <si>
+    <t>about-nci/organization/nci-at-a-glance</t>
+  </si>
+  <si>
+    <t>espanol/match-infantil-infografia</t>
+  </si>
+  <si>
+    <t>reconstruction-fact-sheet</t>
+  </si>
+  <si>
+    <t>March 12, 2016</t>
+  </si>
+  <si>
+    <t>2016-03-12T12:00:00Z</t>
+  </si>
+  <si>
+    <t>2017-07-24T12:00:00Z</t>
+  </si>
+  <si>
+    <t>July 24, 2017</t>
+  </si>
+  <si>
+    <t>about-nci/organization/pediatric-match-infographic</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -223,9 +229,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -543,7 +551,7 @@
   <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="55.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="58.83203125" customWidth="1"/>
     <col min="2" max="2" width="17.1640625" customWidth="1"/>
     <col min="3" max="4" width="14.83203125" customWidth="1"/>
     <col min="5" max="5" width="21.6640625" bestFit="1" customWidth="1"/>
@@ -561,13 +569,13 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="E1" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="F1" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -581,13 +589,13 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
         <v>8</v>
       </c>
       <c r="F2" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -601,13 +609,13 @@
         <v>13</v>
       </c>
       <c r="D3" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
@@ -621,13 +629,13 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
         <v>20</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
@@ -641,18 +649,18 @@
         <v>13</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="E5" t="s">
         <v>22</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>26</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -660,19 +668,19 @@
       <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="D6" t="s">
-        <v>36</v>
-      </c>
-      <c r="E6" t="s">
-        <v>25</v>
+      <c r="D6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>49</v>
       </c>
       <c r="F6" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -681,13 +689,13 @@
         <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
       <c r="F7" t="s">
-        <v>50</v>
+        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -701,18 +709,18 @@
         <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s">
         <v>11</v>
       </c>
       <c r="F8" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B9" t="s">
         <v>7</v>
@@ -721,13 +729,13 @@
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="E9" t="s">
         <v>11</v>
       </c>
       <c r="F9" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -741,13 +749,13 @@
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
         <v>11</v>
       </c>
       <c r="F10" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
@@ -761,33 +769,33 @@
         <v>4</v>
       </c>
       <c r="D11" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B12" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C12" t="s">
         <v>4</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>52</v>
       </c>
       <c r="F12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -800,7 +808,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7CC26DAC-9091-7441-904D-1932A7FF4396}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="63" bestFit="1" customWidth="1"/>
@@ -864,10 +872,10 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B6" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -875,24 +883,35 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
+        <v>37</v>
+      </c>
+      <c r="C8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
         <v>44</v>
       </c>
-      <c r="C8" t="s">
-        <v>4</v>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixed data for missing content
</commit_message>
<xml_diff>
--- a/test-data/dates-data.xlsx
+++ b/test-data/dates-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D6FAC28-9732-F34C-B77F-F9EB14F6658D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA296539-6986-6945-9B90-DD9162259F05}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19140" activeTab="1" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
+    <workbookView xWindow="3620" yWindow="1060" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_simple_dates" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="50">
   <si>
     <t>path</t>
   </si>
@@ -46,9 +46,6 @@
     <t>Cancer Center</t>
   </si>
   <si>
-    <t>about-cancer/coping/feelings/relaxation/loukissas-jen-biography</t>
-  </si>
-  <si>
     <t>Biography</t>
   </si>
   <si>
@@ -179,15 +176,6 @@
   </si>
   <si>
     <t>2016-03-12T12:00:00Z</t>
-  </si>
-  <si>
-    <t>2017-07-24T12:00:00Z</t>
-  </si>
-  <si>
-    <t>July 24, 2017</t>
-  </si>
-  <si>
-    <t>about-nci/organization/pediatric-match-infographic</t>
   </si>
 </sst>
 </file>
@@ -548,7 +536,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61587B9F-5CDD-9140-AFE3-DF7999F08D55}">
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="58.83203125" customWidth="1"/>
@@ -569,18 +557,18 @@
         <v>3</v>
       </c>
       <c r="D1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -589,38 +577,38 @@
         <v>4</v>
       </c>
       <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" t="s">
         <v>25</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B3" t="s">
         <v>2</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" t="s">
         <v>2</v>
@@ -629,38 +617,38 @@
         <v>4</v>
       </c>
       <c r="D4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -669,73 +657,73 @@
         <v>4</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F6" t="s">
         <v>49</v>
-      </c>
-      <c r="F6" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F7" t="s">
         <v>42</v>
-      </c>
-      <c r="F7" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-      <c r="B8" t="s">
-        <v>7</v>
-      </c>
       <c r="C8" t="s">
         <v>4</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E8" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F8" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
       </c>
       <c r="D9" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="E9" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F9" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
@@ -743,63 +731,23 @@
         <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C10" t="s">
         <v>4</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
-      </c>
-      <c r="E10" t="s">
-        <v>11</v>
+        <v>24</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="F10" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
-        <v>24</v>
-      </c>
-      <c r="B11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C11" t="s">
-        <v>4</v>
-      </c>
-      <c r="D11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E11" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F11" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
-        <v>53</v>
-      </c>
-      <c r="B12" t="s">
-        <v>30</v>
-      </c>
-      <c r="C12" t="s">
-        <v>4</v>
-      </c>
-      <c r="D12" t="s">
-        <v>29</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="F12" t="s">
-        <v>51</v>
+        <v>34</v>
       </c>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F12">
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F10">
     <sortCondition ref="B1"/>
   </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -828,7 +776,7 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
@@ -839,7 +787,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
@@ -850,10 +798,10 @@
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B4" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
@@ -861,21 +809,21 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B5" t="s">
         <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -883,21 +831,21 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C8" t="s">
         <v>4</v>
@@ -905,13 +853,13 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B9" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Fixed the data for cross-cuttonig tests that failed on dev enviroanment.
</commit_message>
<xml_diff>
--- a/test-data/dates-data.xlsx
+++ b/test-data/dates-data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/popkhadzeg/eclipse-workspace/cgov-digital-platform-qa/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA296539-6986-6945-9B90-DD9162259F05}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{110C0DAB-F40F-E744-92B2-F4BC34ED67C2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3620" yWindow="1060" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
+    <workbookView xWindow="0" yWindow="460" windowWidth="33600" windowHeight="19140" xr2:uid="{150E7FB9-AAC7-684F-9B42-02331F762CE7}"/>
   </bookViews>
   <sheets>
     <sheet name="pages_with_simple_dates" sheetId="5" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="49">
   <si>
     <t>path</t>
   </si>
@@ -148,15 +148,6 @@
     <t>expectedLabel</t>
   </si>
   <si>
-    <t>espanol/cancer/sobrellevar/sentimientos/hoja-informativa-estres</t>
-  </si>
-  <si>
-    <t>10 de diciembre de 2012</t>
-  </si>
-  <si>
-    <t>2012-12-10T12:00:00Z</t>
-  </si>
-  <si>
     <t>espanol/investigacion/es-hedge-maze</t>
   </si>
   <si>
@@ -169,20 +160,26 @@
     <t>espanol/match-infantil-infografia</t>
   </si>
   <si>
-    <t>reconstruction-fact-sheet</t>
-  </si>
-  <si>
     <t>March 12, 2016</t>
   </si>
   <si>
     <t>2016-03-12T12:00:00Z</t>
+  </si>
+  <si>
+    <t>espanol/hoja-informativa-reconstruccion</t>
+  </si>
+  <si>
+    <t>12 de marzo de 2016</t>
+  </si>
+  <si>
+    <t>types/breast/reconstruction-fact-sheet</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -192,6 +189,14 @@
     </font>
     <font>
       <sz val="12"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -217,11 +222,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -546,23 +552,23 @@
     <col min="6" max="6" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="4" t="s">
         <v>37</v>
       </c>
     </row>
@@ -648,7 +654,7 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>2</v>
@@ -660,15 +666,15 @@
         <v>33</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="F6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="B7" t="s">
         <v>2</v>
@@ -680,10 +686,10 @@
         <v>32</v>
       </c>
       <c r="E7" t="s">
-        <v>41</v>
+        <v>47</v>
       </c>
       <c r="F7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
@@ -763,14 +769,14 @@
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -820,7 +826,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>29</v>
@@ -831,7 +837,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
         <v>29</v>
@@ -842,7 +848,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="B8" t="s">
         <v>36</v>
@@ -853,7 +859,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
         <v>36</v>

</xml_diff>